<commit_message>
some observations in comments
</commit_message>
<xml_diff>
--- a/data/B24_department_schedules_finals/Makine Mühendisliği.xlsx
+++ b/data/B24_department_schedules_finals/Makine Mühendisliği.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ercx2\Desktop\Scheduling Theory_02\Paper\scheduling\Campus-Scheduling\data\department_schedules_finals\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ercx2\Desktop\Scheduling Theory_02\Paper\scheduling\Campus-Scheduling\data\B24_department_schedules_finals\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{92A7EF38-2FF9-4992-9C28-7E93831969F5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CBFC5BDC-0E1B-45B5-9F22-01E689BB4CBA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21100" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>

</xml_diff>